<commit_message>
Catalog audit round 2: true categories from catalog sections, unique images
- Re-derived every category from the catalogs' own section headers: 20 products
  moved (helmet, harnesses, via ferrata, slings, crash pad, quickdraw sets,
  screwlinks, Warp->Pulleys, new Rope Clamps & Ascenders; Voltage III ->
  Performance). 17 categories now mirror the catalog structure.
- Fixed 22 duplicate-image groups via per-page 1:1 photo<->article assignment;
  97 images re-extracted (one genuine shared photo remains: Screwlink 8/10mm)
- Replaced bogus 8271 (Kiwi-page clone) with real 88271 Axiom; Bud -> Belay
  Devices with correct figure-8 photo; Ohmega description trimmed to source;
  RFID inferred specs moved to attributes
- Audit: 100% of descriptions/features and 780/781 specs traceable to source
- docs/AUDIT-REPORT.md + regenerated catalog-review.xlsx, products.ts, seed.sql

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/catalog-review.xlsx
+++ b/docs/catalog-review.xlsx
@@ -656,7 +656,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Chalk Bags</t>
+          <t>Belay Devices</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -733,7 +733,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Chalk Bags</t>
+          <t>Crash Pads</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Chalk &amp; Accessories</t>
+          <t>Harnesses</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1755,7 +1755,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Chalk &amp; Accessories</t>
+          <t>Harnesses</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1832,7 +1832,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Chalk &amp; Accessories</t>
+          <t>Via Ferrata</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1909,7 +1909,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Chalk &amp; Accessories</t>
+          <t>Carabiners &amp; Quickdraws</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1986,7 +1986,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Chalk &amp; Accessories</t>
+          <t>Carabiners &amp; Quickdraws</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2059,7 +2059,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Chalk &amp; Accessories</t>
+          <t>Carabiners &amp; Quickdraws</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2132,7 +2132,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Chalk &amp; Accessories</t>
+          <t>Carabiners &amp; Quickdraws</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2667,7 +2667,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Hardware Accessories</t>
+          <t>Pulleys</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2817,7 +2817,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Hardware Accessories</t>
+          <t>Rope Clamps &amp; Ascenders</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2894,7 +2894,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Hardware Accessories</t>
+          <t>Rope Clamps &amp; Ascenders</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3223,7 +3223,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>Rethink belaying - weighing in at barely 190 g, the compact OHMEGA is a highly versatile brake assistant suitable for use by a wide target group. Whether in climbing gyms, at the crag, or on alpine sport climbing routes (when using a single rope), it offers genuine added value in terms of safety and comfort for both climbers and belayers. This benefits beginners, experienced climbers, and pros as well as rope parties with and without a weight difference. The integrated HMPE sling enables users to switch between three different braking levels with a simple hand movement to suit the weight distribution. The integrated pulley keeps the friction generated at the first bolt lower than when using a quickdraw, so users won't notice the OHMEGA when climbing or clipping, even on long and difficult routes. Thanks to the short HMPE sling and the resultant minimal activation distance, the belayer finds it easier to belay dynamically and softly, reducing the risk of impact-induced injuries. In the event of a fall, the cam brakes the fall, supporting the belayer and balancing out weight differences. As a result, the belayer won't be pulled off the ground in the event of a big fall. With falls from a low height, the braking effect of the OHMEGA reduces the risk of both the climbing partners colliding and the climber hitting the ground. The OHMEGA also brakes reliably if the climber falls into the device. Simple, light, and offering enhanced safety and comfort for both climbing partners, the OHMEGA opens up new possibilities and makes belaying a completely new experience.</t>
+          <t>Rethink belaying - weighing in at barely 190 g, the compact OHMEGA is a highly versatile brake assistant suitable for use by a wide target group. Whether in climbing gyms, at the crag, or on alpine sport climbing routes (when using a single rope), it offers genuine added value in terms of safety and comfort for both climbers and belayers. This benefits beginners, experienced climbers, and pros as well as rope parties with and without a weight difference. The integrated HMPE sling enables users to switch between three different braking levels with a simple hand movement to suit the weight distribution. The integrated pulley keeps the friction generated at the first bolt lower than when using a quickdraw, so users won't notice the OHMEGA when climbing or clipping, even on long and difficult routes. Thanks to the short HMPE sling and the resultant minimal activation distance, the belayer finds it easier to belay dynamically and softly, reducing the risk of impact-induced injuries. In the event of a fall, the cam brakes the fall, supporting the belayer and balancing out weight differences. As a result, the belayer won't be pulled off the ground in the event of a big fall. With falls from a low height, the braking effect of the OHMEGA reduces the risk of both the climbing partners colliding and the climber hitting the ground.</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -3315,18 +3315,22 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>8271</t>
+          <t>88271</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
+          <t>Axiom (client list wrote 8271 — missing digit)</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
           <t>Axiom</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Kiwi</t>
+          <t>Axiom</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -3336,7 +3340,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Belay Devices</t>
+          <t>Carabiners &amp; Quickdraws</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -3349,7 +3353,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>56 g</t>
+          <t>66g</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -3359,27 +3363,27 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>icemint 329, night 017, oasis 138</t>
+          <t>icemint 329</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>/images/products/8271.webp</t>
+          <t>/images/products/88271.webp</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>Light and compact oval carabiner. The oval shape optimally distributes the load on the longitudinal axis and offers a large capacity. The ideal carabiner for clearly organized gear.</t>
+          <t>Carabiner with integrated pulley in the spine. The pulley reduces rope friction to a minimum and maintains its function even under load. The optimized design of the AXIOM ensures that the rope is always ideally guided so that it can always run on the pulley. Available with a classic gate or the automatic and very compact Slider locking gate. The gate opens on the pulley side, which makes installing the rope easier.</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>Keylock closure mechanism for optimum handling when clipping and unclipping | Available as a gate or slider version</t>
+          <t>Very lightweight construction | Available as a gate or slider version | Pulley maintains its function even under load | Optimized design for perfect rope guidance in the carabiner at all times | Efficiency: 86 %</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>Certification: EN 12275 | Material: Aluminium | Closure: Normal | Carabiner shape: Oval | Fmax. major axis: 24 kN | Fmax. open: 8 kN | Fmax. minor axis: 10 kN | Width: 57 mm | Length: 100 mm | Gate opening: 23 mm | Weight: 56 g</t>
+          <t>Certification: EN 12275 | Material: Aluminium | Closure: Normal | Carabiner shape: Axiom | Fmax. major axis: 22 kN | Fmax. open: 7 kN | Fmax. minor axis: 8 kN | Width: 65 mm | Length: 100 mm | Gate opening: 18 mm | Weight: 66g</t>
         </is>
       </c>
       <c r="P39" t="inlineStr"/>
@@ -3413,7 +3417,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Chalk &amp; Accessories</t>
+          <t>Carabiners &amp; Quickdraws</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -3490,7 +3494,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Chalk &amp; Accessories</t>
+          <t>Carabiners &amp; Quickdraws</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -3567,7 +3571,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Chalk &amp; Accessories</t>
+          <t>Slings &amp; Webbing</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -3640,7 +3644,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Chalk &amp; Accessories</t>
+          <t>Carabiners &amp; Quickdraws</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -3979,7 +3983,7 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>Certification: EN 362; EN 12275 H | Material: Aluminium | Closure: Screw | RFID: Yes | Carabiner shape: HMS | Fmax. major axis: 26 kN | Fmax. open: 9 kN | Fmax. minor axis: 10 kN | Width: 75 mm | Length: 110 mm | Gate opening: 24 mm | Weight: 74g</t>
+          <t>Certification: EN 362; EN 12275 H | Material: Aluminium | Closure: Screw | Carabiner shape: HMS | Fmax. major axis: 26 kN | Fmax. open: 9 kN | Fmax. minor axis: 10 kN | Width: 75 mm | Length: 110 mm | Gate opening: 24 mm | Weight: 74g</t>
         </is>
       </c>
       <c r="P47" t="inlineStr"/>
@@ -4056,7 +4060,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>Certification: EN 362; EN 12275 H | Material: Aluminium | Closure: Triple | RFID: Yes | Carabiner shape: HMS | Fmax. major axis: 26 kN | Fmax. open: 9 kN | Fmax. minor axis: 10 kN | Width: 75 mm | Length: 110 mm | Gate opening: 24 mm | Weight: 74g</t>
+          <t>Certification: EN 362; EN 12275 H | Material: Aluminium | Closure: Triple | Carabiner shape: HMS | Fmax. major axis: 26 kN | Fmax. open: 9 kN | Fmax. minor axis: 10 kN | Width: 75 mm | Length: 110 mm | Gate opening: 24 mm | Weight: 74g</t>
         </is>
       </c>
       <c r="P48" t="inlineStr"/>
@@ -6230,7 +6234,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Helmets</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -6611,7 +6615,7 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Descenders &amp; Rescue</t>
+          <t>Rope Clamps &amp; Ascenders</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -6684,7 +6688,7 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Descenders &amp; Rescue</t>
+          <t>Hardware Accessories</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -6761,7 +6765,7 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Spare Parts</t>
+          <t>Hardware Accessories</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -7053,7 +7057,7 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Climbing Shoes — High-End</t>
+          <t>Climbing Shoes — Performance</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">

</xml_diff>

<commit_message>
Client-final catalog (96 items, 12 categories) + real Legal/Compliance pages
- Categories now exactly match the client's authoritative list; removed Giga Jul
  & Mega Jul II (not requested). Ultralight Junior III moved Carabiners -> Helmets.
  Verified: site set == client list (96), no extras/dupes.
- Real footer pages (wouter routes /certifications /privacy /terms /returns),
  replacing dead "#" links. Content drafted from source facts:
  * Certifications & Compliance: accurate CE (PPE Reg 2016/425) + UIAA standards,
    framed correctly (Cliffhanger supplies gear certified by Edelrid/Tendon) -
    a real E-E-A-T / GEO trust page
  * Privacy / Terms / Returns: honest, Lebanon-specific, with [PLACEHOLDER]s the
    client must fill (company entity, dates, return window)
- SPA fallback (vercel rewrite + netlify _redirects), sitemap now lists the pages

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/catalog-review.xlsx
+++ b/docs/catalog-review.xlsx
@@ -733,7 +733,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Crash Pads</t>
+          <t>Chalk Bags</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1390,7 +1390,7 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Chalk &amp; Accessories</t>
+          <t>Chalk Bags</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1463,7 +1463,7 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Chalk &amp; Accessories</t>
+          <t>Chalk Bags</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
@@ -1536,7 +1536,7 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Chalk &amp; Accessories</t>
+          <t>Chalk Bags</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
@@ -1609,7 +1609,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Chalk &amp; Accessories</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Harnesses</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1755,7 +1755,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Harnesses</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1832,7 +1832,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Via Ferrata</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1909,7 +1909,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1986,7 +1986,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2059,7 +2059,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2132,7 +2132,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2667,7 +2667,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Pulleys</t>
+          <t>Hardware Accessories</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2817,7 +2817,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Rope Clamps &amp; Ascenders</t>
+          <t>Hardware Accessories</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2894,7 +2894,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Rope Clamps &amp; Ascenders</t>
+          <t>Hardware Accessories</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3340,7 +3340,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Carabiners</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -3417,7 +3417,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Carabiners</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -3494,7 +3494,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Carabiners</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -3571,7 +3571,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Slings &amp; Webbing</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -3644,7 +3644,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Accessories</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -3709,7 +3709,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Carabiners</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -3786,7 +3786,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Carabiners</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Carabiners</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -3940,7 +3940,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Carabiners</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -4017,7 +4017,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Carabiners</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -4094,7 +4094,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Carabiners</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -4171,7 +4171,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Carabiners</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -4248,7 +4248,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Carabiners</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -4325,7 +4325,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Carabiners</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -4402,7 +4402,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Carabiners</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -4479,7 +4479,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Carabiners</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -4556,7 +4556,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Carabiners</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -4633,7 +4633,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Carabiners</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -4710,7 +4710,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Carabiners</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -4787,7 +4787,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Carabiners</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -4864,7 +4864,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Carabiners</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -4941,7 +4941,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Carabiners</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -5018,7 +5018,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Carabiners</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -5095,7 +5095,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Carabiners</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -5172,7 +5172,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Carabiners</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -5249,7 +5249,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Carabiners</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -5326,7 +5326,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Carabiners</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -5403,7 +5403,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Carabiners</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -5480,7 +5480,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Carabiners</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -5557,7 +5557,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Carabiners</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -5634,7 +5634,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Carabiners</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -5711,7 +5711,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Carabiners</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -5788,7 +5788,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Carabiners</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -5865,7 +5865,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Carabiners</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -5942,7 +5942,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Carabiners</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -6003,7 +6003,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Carabiners</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -6080,7 +6080,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Carabiners</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -6157,7 +6157,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Carabiners &amp; Quickdraws</t>
+          <t>Carabiners</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -6301,7 +6301,7 @@
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>Giga Jul</t>
+          <t>NOT ON SITE</t>
         </is>
       </c>
       <c r="E78" s="4" t="inlineStr">
@@ -6309,11 +6309,7 @@
           <t>CHECK — request ambiguous</t>
         </is>
       </c>
-      <c r="F78" s="3" t="inlineStr">
-        <is>
-          <t>Belay Devices</t>
-        </is>
-      </c>
+      <c r="F78" s="3" t="inlineStr"/>
       <c r="G78" s="3" t="inlineStr">
         <is>
           <t>DWB_Sport_2026_EN-1.pdf</t>
@@ -6322,41 +6318,13 @@
       <c r="H78" s="3" t="n">
         <v>163</v>
       </c>
-      <c r="I78" s="3" t="inlineStr">
-        <is>
-          <t>121 g</t>
-        </is>
-      </c>
-      <c r="J78" s="3" t="inlineStr">
-        <is>
-          <t>EN 15151-2</t>
-        </is>
-      </c>
-      <c r="K78" s="3" t="inlineStr">
-        <is>
-          <t>slate 663</t>
-        </is>
-      </c>
-      <c r="L78" s="3" t="inlineStr">
-        <is>
-          <t>/images/products/73742.webp</t>
-        </is>
-      </c>
-      <c r="M78" s="3" t="inlineStr">
-        <is>
-          <t>The most versatile ever belay device. The GIGA JUL is a standard and assisted braking tuber in one. The assisted braking function which supports the braking force can be activated or disabled by an intelligent mechanism. For situation-dependent belaying and abseiling, especially in alpine terrain.</t>
-        </is>
-      </c>
-      <c r="N78" s="3" t="inlineStr">
-        <is>
-          <t>Small eyelet for releasing unit with a carabiner when bringing up your partner | Suitable for 7.1–10.0 mm ropes | Intelligent hybrid design: body made of ultra-light aluminum, areas susceptible to abrasion made of robust stainless steel | Guide mode: simple and rapid abseiling and bringing up seconds plus comfortable belaying from a belay station as a doubled rope | Assisted braking guide mode: brake boost for catching falls in leader mode | Rope can be paid out faster in assisted braking guide mode by holding the device in the 'open' position with the thumb</t>
-        </is>
-      </c>
-      <c r="O78" s="3" t="inlineStr">
-        <is>
-          <t>Certification: EN 15151-2 | Material: Steel, Polyamide | Approved rope diameter: 7.1–10 mm | Weight: 121 g</t>
-        </is>
-      </c>
+      <c r="I78" s="3" t="inlineStr"/>
+      <c r="J78" s="3" t="inlineStr"/>
+      <c r="K78" s="3" t="inlineStr"/>
+      <c r="L78" s="3" t="inlineStr"/>
+      <c r="M78" s="3" t="inlineStr"/>
+      <c r="N78" s="3" t="inlineStr"/>
+      <c r="O78" s="3" t="inlineStr"/>
       <c r="P78" s="3" t="inlineStr"/>
       <c r="Q78" s="3" t="inlineStr"/>
     </row>
@@ -6378,7 +6346,7 @@
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>Mega Jul II</t>
+          <t>NOT ON SITE</t>
         </is>
       </c>
       <c r="E79" s="4" t="inlineStr">
@@ -6386,11 +6354,7 @@
           <t>CHECK — request ambiguous</t>
         </is>
       </c>
-      <c r="F79" s="3" t="inlineStr">
-        <is>
-          <t>Belay Devices</t>
-        </is>
-      </c>
+      <c r="F79" s="3" t="inlineStr"/>
       <c r="G79" s="3" t="inlineStr">
         <is>
           <t>DWB_Sport_2026_EN-1.pdf</t>
@@ -6399,41 +6363,13 @@
       <c r="H79" s="3" t="n">
         <v>163</v>
       </c>
-      <c r="I79" s="3" t="inlineStr">
-        <is>
-          <t>75 g</t>
-        </is>
-      </c>
-      <c r="J79" s="3" t="inlineStr">
-        <is>
-          <t>EN 15151-2</t>
-        </is>
-      </c>
-      <c r="K79" s="3" t="inlineStr">
-        <is>
-          <t>slate 663</t>
-        </is>
-      </c>
-      <c r="L79" s="3" t="inlineStr">
-        <is>
-          <t>/images/products/73831.webp</t>
-        </is>
-      </c>
-      <c r="M79" s="3" t="inlineStr">
-        <is>
-          <t>Our versatile, lightweight, and durable stainless steel belay device and descender.</t>
-        </is>
-      </c>
-      <c r="N79" s="3" t="inlineStr">
-        <is>
-          <t>Robust solid stainless steel construction | The increased braking effect of the new device geometry assists the belayer when arresting a fall as a leader | Faster rope payout when lead climbing thanks to the thumb-loop-based operation | Additional eyelet for unlocking the device in follower mode using a carabiner | Suitable for ropes with a diameter of 7.8 to 10.0 mm | Suitable for belaying a leader, bringing up one or two followers, and rappelling</t>
-        </is>
-      </c>
-      <c r="O79" s="3" t="inlineStr">
-        <is>
-          <t>Certification: EN 15151-2 | Material: Steel | Approved rope diameter: 7.8–10.0 mm | Weight: 75 g</t>
-        </is>
-      </c>
+      <c r="I79" s="3" t="inlineStr"/>
+      <c r="J79" s="3" t="inlineStr"/>
+      <c r="K79" s="3" t="inlineStr"/>
+      <c r="L79" s="3" t="inlineStr"/>
+      <c r="M79" s="3" t="inlineStr"/>
+      <c r="N79" s="3" t="inlineStr"/>
+      <c r="O79" s="3" t="inlineStr"/>
       <c r="P79" s="3" t="inlineStr"/>
       <c r="Q79" s="3" t="inlineStr"/>
     </row>
@@ -6615,7 +6551,7 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Rope Clamps &amp; Ascenders</t>
+          <t>Descenders &amp; Rescue</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -6688,7 +6624,7 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Hardware Accessories</t>
+          <t>Descenders &amp; Rescue</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -6765,7 +6701,7 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Hardware Accessories</t>
+          <t>Spare Parts</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -7057,7 +6993,7 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Climbing Shoes — Performance</t>
+          <t>Climbing Shoes — High-End</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">

</xml_diff>